<commit_message>
feat(viceri-study): publish specification and test suite v1.2
</commit_message>
<xml_diff>
--- a/output/xlsx/AdministradorEditaTerminal--GT-.xlsx
+++ b/output/xlsx/AdministradorEditaTerminal--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="61">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 7 test case(s)</t>
+    <t>Size: 8 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -171,6 +171,15 @@
   </si>
   <si>
     <t>TC7</t>
+  </si>
+  <si>
+    <t>Alternative Flow 6: Volta para tela inicial de sistema</t>
+  </si>
+  <si>
+    <t>Administrador: clica no botao Voltar</t>
+  </si>
+  <si>
+    <t>TC8</t>
   </si>
   <si>
     <t>Exception Flow 1: Usuario nao preenche algum campo obrigatorio</t>
@@ -277,7 +286,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
@@ -1251,13 +1260,13 @@
         <v>2.0</v>
       </c>
       <c r="B77" t="s" s="3">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C77" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D77" t="s" s="3">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E77" t="s" s="3">
         <v>27</v>
@@ -1271,13 +1280,13 @@
         <v>3.0</v>
       </c>
       <c r="B78" t="s" s="3">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C78" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D78" t="s" s="3">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="E78" t="s" s="3">
         <v>27</v>
@@ -1291,13 +1300,13 @@
         <v>4.0</v>
       </c>
       <c r="B79" t="s" s="3">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="C79" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D79" t="s" s="3">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="E79" t="s" s="3">
         <v>27</v>
@@ -1311,7 +1320,148 @@
         <v>33</v>
       </c>
       <c r="B80" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C83" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E83" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="E84" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B86" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C86" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D86" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E86" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F86" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B87" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C87" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D87" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E87" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F87" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B88" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C88" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D88" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E88" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F88" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B89" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="C89" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D89" t="s" s="3">
         <v>57</v>
+      </c>
+      <c r="E89" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F89" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B90" t="s" s="3">
+        <v>58</v>
+      </c>
+      <c r="C90" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D90" t="s" s="3">
+        <v>59</v>
+      </c>
+      <c r="E90" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F90" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>